<commit_message>
Nuova pagina Allestimenti (wrapping/vetrine/stand/eventi) + card carousel
- allestimenti.html: hero, valore, galleria realizzazioni filtrabile + lightbox, processo, CTA
- js/allestimenti.js (dati segnaposto), riuso stili maxi.css
- card SVG nel carousel home -> allestimenti.html
- voce di menu 'Allestimenti' + link footer su tutte le pagine (IT/EN/ZH)
- sitemap, schema Service+Breadcrumb, cartella assets/foto/allestimenti

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/maxi-impianti.xlsx
+++ b/maxi-impianti.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MSI\Documents\CLAUDE\Projects\SCHEDE IMPIANTI DI AFFISSIONE\sito-diessemedia\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73BD18ED-1CE7-4DE9-A61C-3E234D450908}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD9667E9-0BE2-418A-A555-8064A4A15D13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,12 +16,25 @@
     <sheet name="Impianti" sheetId="1" r:id="rId1"/>
     <sheet name="Istruzioni" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="179">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="281" uniqueCount="178">
   <si>
     <t>code</t>
   </si>
@@ -99,9 +112,6 @@
   </si>
   <si>
     <t>mx-na-01.jpg</t>
-  </si>
-  <si>
-    <t>Ponteggio</t>
   </si>
   <si>
     <t>mx-na-02.jpg</t>
@@ -1169,7 +1179,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K30"/>
+  <dimension ref="A1:K31"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11" customWidth="1"/>
@@ -1256,89 +1266,89 @@
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>22</v>
       </c>
       <c r="C3" s="12" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="E3" s="15" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F3" s="3">
         <v>36</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="I3" s="3" t="s">
         <v>25</v>
       </c>
       <c r="J3" s="9" t="s">
+        <v>121</v>
+      </c>
+      <c r="K3" s="17" t="s">
         <v>122</v>
-      </c>
-      <c r="K3" s="17" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>22</v>
       </c>
       <c r="C4" s="12" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E4" s="15" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F4" s="3">
         <v>36</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="J4" s="9" t="s">
+        <v>123</v>
+      </c>
+      <c r="K4" s="17" t="s">
         <v>124</v>
-      </c>
-      <c r="K4" s="17" t="s">
-        <v>125</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>22</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="E5" s="15" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F5" s="3">
         <v>70</v>
@@ -1347,31 +1357,31 @@
         <v>24</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="I5" s="3"/>
       <c r="J5" s="18" t="s">
+        <v>125</v>
+      </c>
+      <c r="K5" s="19" t="s">
         <v>126</v>
-      </c>
-      <c r="K5" s="19" t="s">
-        <v>127</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>22</v>
       </c>
       <c r="C6" s="12" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="E6" s="15" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F6" s="3">
         <v>70</v>
@@ -1380,28 +1390,31 @@
         <v>24</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="I6" s="3"/>
       <c r="J6" s="18" t="s">
+        <v>127</v>
+      </c>
+      <c r="K6" s="19" t="s">
         <v>128</v>
-      </c>
-      <c r="K6" s="19" t="s">
-        <v>129</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>22</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>82</v>
+        <v>81</v>
+      </c>
+      <c r="D7" s="30" t="s">
+        <v>23</v>
       </c>
       <c r="E7" s="15" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F7" s="29">
         <v>36</v>
@@ -1410,24 +1423,27 @@
         <v>24</v>
       </c>
       <c r="J7" s="18" t="s">
+        <v>129</v>
+      </c>
+      <c r="K7" s="19" t="s">
         <v>130</v>
-      </c>
-      <c r="K7" s="19" t="s">
-        <v>131</v>
       </c>
     </row>
     <row r="8" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>22</v>
       </c>
       <c r="C8" s="12" t="s">
-        <v>83</v>
+        <v>82</v>
+      </c>
+      <c r="D8" s="30" t="s">
+        <v>23</v>
       </c>
       <c r="E8" s="15" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F8" s="29">
         <v>70</v>
@@ -1436,24 +1452,27 @@
         <v>24</v>
       </c>
       <c r="J8" s="18" t="s">
+        <v>131</v>
+      </c>
+      <c r="K8" s="19" t="s">
         <v>132</v>
-      </c>
-      <c r="K8" s="19" t="s">
-        <v>133</v>
       </c>
     </row>
     <row r="9" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>22</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>84</v>
+        <v>83</v>
+      </c>
+      <c r="D9" s="30" t="s">
+        <v>23</v>
       </c>
       <c r="E9" s="15" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F9" s="29">
         <v>70</v>
@@ -1462,24 +1481,27 @@
         <v>24</v>
       </c>
       <c r="J9" s="20" t="s">
+        <v>133</v>
+      </c>
+      <c r="K9" s="21" t="s">
         <v>134</v>
-      </c>
-      <c r="K9" s="21" t="s">
-        <v>135</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>22</v>
       </c>
       <c r="C10" s="12" t="s">
-        <v>85</v>
+        <v>84</v>
+      </c>
+      <c r="D10" s="30" t="s">
+        <v>23</v>
       </c>
       <c r="E10" s="15" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F10" s="29">
         <v>36</v>
@@ -1488,24 +1510,27 @@
         <v>24</v>
       </c>
       <c r="J10" s="20" t="s">
+        <v>135</v>
+      </c>
+      <c r="K10" s="21" t="s">
         <v>136</v>
-      </c>
-      <c r="K10" s="21" t="s">
-        <v>137</v>
       </c>
     </row>
     <row r="11" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>22</v>
       </c>
       <c r="C11" s="12" t="s">
-        <v>86</v>
+        <v>85</v>
+      </c>
+      <c r="D11" s="30" t="s">
+        <v>23</v>
       </c>
       <c r="E11" s="15" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F11" s="29">
         <v>70</v>
@@ -1514,24 +1539,27 @@
         <v>24</v>
       </c>
       <c r="J11" s="18" t="s">
+        <v>137</v>
+      </c>
+      <c r="K11" s="19" t="s">
         <v>138</v>
-      </c>
-      <c r="K11" s="19" t="s">
-        <v>139</v>
       </c>
     </row>
     <row r="12" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>22</v>
       </c>
       <c r="C12" s="12" t="s">
-        <v>87</v>
+        <v>86</v>
+      </c>
+      <c r="D12" s="30" t="s">
+        <v>23</v>
       </c>
       <c r="E12" s="15" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F12" s="29">
         <v>49</v>
@@ -1540,24 +1568,27 @@
         <v>24</v>
       </c>
       <c r="J12" s="18" t="s">
+        <v>139</v>
+      </c>
+      <c r="K12" s="19" t="s">
         <v>140</v>
-      </c>
-      <c r="K12" s="19" t="s">
-        <v>141</v>
       </c>
     </row>
     <row r="13" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>22</v>
       </c>
       <c r="C13" s="13" t="s">
-        <v>88</v>
+        <v>87</v>
+      </c>
+      <c r="D13" s="30" t="s">
+        <v>23</v>
       </c>
       <c r="E13" s="15" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F13" s="29">
         <v>50</v>
@@ -1566,24 +1597,27 @@
         <v>24</v>
       </c>
       <c r="J13" s="9" t="s">
+        <v>141</v>
+      </c>
+      <c r="K13" s="17" t="s">
         <v>142</v>
-      </c>
-      <c r="K13" s="17" t="s">
-        <v>143</v>
       </c>
     </row>
     <row r="14" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" s="7" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>22</v>
       </c>
       <c r="C14" s="13" t="s">
-        <v>89</v>
+        <v>88</v>
+      </c>
+      <c r="D14" s="30" t="s">
+        <v>23</v>
       </c>
       <c r="E14" s="15" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F14" s="29">
         <v>70</v>
@@ -1592,24 +1626,27 @@
         <v>24</v>
       </c>
       <c r="J14" s="9" t="s">
+        <v>143</v>
+      </c>
+      <c r="K14" s="17" t="s">
         <v>144</v>
-      </c>
-      <c r="K14" s="17" t="s">
-        <v>145</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B15" s="3" t="s">
         <v>22</v>
       </c>
       <c r="C15" s="13" t="s">
-        <v>90</v>
+        <v>89</v>
+      </c>
+      <c r="D15" s="30" t="s">
+        <v>23</v>
       </c>
       <c r="E15" s="15" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F15" s="29">
         <v>48</v>
@@ -1618,24 +1655,27 @@
         <v>24</v>
       </c>
       <c r="J15" s="9" t="s">
+        <v>145</v>
+      </c>
+      <c r="K15" s="17" t="s">
         <v>146</v>
-      </c>
-      <c r="K15" s="17" t="s">
-        <v>147</v>
       </c>
     </row>
     <row r="16" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B16" s="3" t="s">
         <v>22</v>
       </c>
       <c r="C16" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
+      </c>
+      <c r="D16" s="30" t="s">
+        <v>23</v>
       </c>
       <c r="E16" s="15" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F16" s="29">
         <v>50</v>
@@ -1644,24 +1684,27 @@
         <v>24</v>
       </c>
       <c r="J16" s="9" t="s">
+        <v>147</v>
+      </c>
+      <c r="K16" s="17" t="s">
         <v>148</v>
-      </c>
-      <c r="K16" s="17" t="s">
-        <v>149</v>
       </c>
     </row>
     <row r="17" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A17" s="9" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>22</v>
       </c>
       <c r="C17" s="13" t="s">
-        <v>92</v>
+        <v>91</v>
+      </c>
+      <c r="D17" s="30" t="s">
+        <v>23</v>
       </c>
       <c r="E17" s="15" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F17" s="29">
         <v>70</v>
@@ -1670,24 +1713,27 @@
         <v>24</v>
       </c>
       <c r="J17" s="9" t="s">
+        <v>149</v>
+      </c>
+      <c r="K17" s="17" t="s">
         <v>150</v>
-      </c>
-      <c r="K17" s="17" t="s">
-        <v>151</v>
       </c>
     </row>
     <row r="18" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="10" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B18" s="3" t="s">
         <v>22</v>
       </c>
       <c r="C18" s="13" t="s">
-        <v>93</v>
+        <v>92</v>
+      </c>
+      <c r="D18" s="30" t="s">
+        <v>23</v>
       </c>
       <c r="E18" s="15" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F18" s="29">
         <v>70</v>
@@ -1696,24 +1742,27 @@
         <v>24</v>
       </c>
       <c r="J18" s="9" t="s">
+        <v>151</v>
+      </c>
+      <c r="K18" s="17" t="s">
         <v>152</v>
-      </c>
-      <c r="K18" s="17" t="s">
-        <v>153</v>
       </c>
     </row>
     <row r="19" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A19" s="9" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>22</v>
       </c>
       <c r="C19" s="13" t="s">
-        <v>94</v>
+        <v>93</v>
+      </c>
+      <c r="D19" s="30" t="s">
+        <v>23</v>
       </c>
       <c r="E19" s="15" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F19" s="29">
         <v>50</v>
@@ -1722,24 +1771,27 @@
         <v>24</v>
       </c>
       <c r="J19" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="K19" s="17" t="s">
         <v>154</v>
-      </c>
-      <c r="K19" s="17" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" s="9" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B20" s="3" t="s">
         <v>22</v>
       </c>
       <c r="C20" s="13" t="s">
-        <v>95</v>
+        <v>94</v>
+      </c>
+      <c r="D20" s="30" t="s">
+        <v>23</v>
       </c>
       <c r="E20" s="15" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="F20" s="29">
         <v>40</v>
@@ -1748,24 +1800,27 @@
         <v>24</v>
       </c>
       <c r="J20" s="9" t="s">
+        <v>155</v>
+      </c>
+      <c r="K20" s="17" t="s">
         <v>156</v>
-      </c>
-      <c r="K20" s="17" t="s">
-        <v>157</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" s="9" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B21" s="3" t="s">
         <v>22</v>
       </c>
       <c r="C21" s="13" t="s">
-        <v>96</v>
+        <v>95</v>
+      </c>
+      <c r="D21" s="30" t="s">
+        <v>23</v>
       </c>
       <c r="E21" s="15" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F21" s="29">
         <v>63</v>
@@ -1774,24 +1829,27 @@
         <v>24</v>
       </c>
       <c r="J21" s="9" t="s">
+        <v>157</v>
+      </c>
+      <c r="K21" s="17" t="s">
         <v>158</v>
-      </c>
-      <c r="K21" s="17" t="s">
-        <v>159</v>
       </c>
     </row>
     <row r="22" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A22" s="9" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B22" s="3" t="s">
         <v>22</v>
       </c>
       <c r="C22" s="13" t="s">
-        <v>97</v>
+        <v>96</v>
+      </c>
+      <c r="D22" s="30" t="s">
+        <v>23</v>
       </c>
       <c r="E22" s="15" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F22" s="29">
         <v>36</v>
@@ -1800,24 +1858,27 @@
         <v>24</v>
       </c>
       <c r="J22" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="K22" s="17" t="s">
         <v>160</v>
-      </c>
-      <c r="K22" s="17" t="s">
-        <v>161</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" s="9" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B23" s="3" t="s">
         <v>22</v>
       </c>
       <c r="C23" s="13" t="s">
-        <v>98</v>
+        <v>97</v>
+      </c>
+      <c r="D23" s="30" t="s">
+        <v>23</v>
       </c>
       <c r="E23" s="15" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="F23" s="29">
         <v>48</v>
@@ -1826,24 +1887,27 @@
         <v>24</v>
       </c>
       <c r="J23" s="9" t="s">
+        <v>161</v>
+      </c>
+      <c r="K23" s="17" t="s">
         <v>162</v>
-      </c>
-      <c r="K23" s="17" t="s">
-        <v>163</v>
       </c>
     </row>
     <row r="24" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A24" s="11" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B24" s="3" t="s">
         <v>22</v>
       </c>
       <c r="C24" s="13" t="s">
-        <v>99</v>
+        <v>98</v>
+      </c>
+      <c r="D24" s="30" t="s">
+        <v>23</v>
       </c>
       <c r="E24" s="15" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F24" s="29">
         <v>96</v>
@@ -1852,24 +1916,27 @@
         <v>24</v>
       </c>
       <c r="J24" s="9" t="s">
+        <v>163</v>
+      </c>
+      <c r="K24" s="17" t="s">
         <v>164</v>
-      </c>
-      <c r="K24" s="17" t="s">
-        <v>165</v>
       </c>
     </row>
     <row r="25" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A25" s="9" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B25" s="3" t="s">
         <v>22</v>
       </c>
       <c r="C25" s="13" t="s">
-        <v>100</v>
+        <v>99</v>
+      </c>
+      <c r="D25" s="30" t="s">
+        <v>23</v>
       </c>
       <c r="E25" s="15" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F25" s="29">
         <v>112</v>
@@ -1878,24 +1945,27 @@
         <v>24</v>
       </c>
       <c r="J25" s="22" t="s">
+        <v>165</v>
+      </c>
+      <c r="K25" s="23" t="s">
         <v>166</v>
-      </c>
-      <c r="K25" s="23" t="s">
-        <v>167</v>
       </c>
     </row>
     <row r="26" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A26" s="9" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B26" s="3" t="s">
         <v>22</v>
       </c>
       <c r="C26" s="13" t="s">
-        <v>101</v>
+        <v>100</v>
+      </c>
+      <c r="D26" s="30" t="s">
+        <v>23</v>
       </c>
       <c r="E26" s="15" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F26" s="29">
         <v>112</v>
@@ -1904,10 +1974,10 @@
         <v>24</v>
       </c>
       <c r="J26" s="22" t="s">
+        <v>167</v>
+      </c>
+      <c r="K26" s="23" t="s">
         <v>168</v>
-      </c>
-      <c r="K26" s="23" t="s">
-        <v>169</v>
       </c>
     </row>
     <row r="27" spans="1:11" ht="30" x14ac:dyDescent="0.25">
@@ -1916,10 +1986,13 @@
         <v>22</v>
       </c>
       <c r="C27" s="13" t="s">
-        <v>102</v>
+        <v>101</v>
+      </c>
+      <c r="D27" s="30" t="s">
+        <v>23</v>
       </c>
       <c r="E27" s="15" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F27" s="29">
         <v>70</v>
@@ -1928,10 +2001,10 @@
         <v>24</v>
       </c>
       <c r="J27" s="24" t="s">
+        <v>169</v>
+      </c>
+      <c r="K27" s="25" t="s">
         <v>170</v>
-      </c>
-      <c r="K27" s="25" t="s">
-        <v>171</v>
       </c>
     </row>
     <row r="28" spans="1:11" ht="30" x14ac:dyDescent="0.25">
@@ -1940,10 +2013,13 @@
         <v>22</v>
       </c>
       <c r="C28" s="13" t="s">
-        <v>103</v>
+        <v>102</v>
+      </c>
+      <c r="D28" s="30" t="s">
+        <v>23</v>
       </c>
       <c r="E28" s="15" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F28" s="29">
         <v>32</v>
@@ -1952,24 +2028,27 @@
         <v>24</v>
       </c>
       <c r="J28" s="24" t="s">
+        <v>171</v>
+      </c>
+      <c r="K28" s="25" t="s">
         <v>172</v>
-      </c>
-      <c r="K28" s="25" t="s">
-        <v>173</v>
       </c>
     </row>
     <row r="29" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A29" s="9" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B29" s="3" t="s">
         <v>22</v>
       </c>
       <c r="C29" s="13" t="s">
-        <v>104</v>
+        <v>103</v>
+      </c>
+      <c r="D29" s="30" t="s">
+        <v>23</v>
       </c>
       <c r="E29" s="15" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F29" s="29">
         <v>50</v>
@@ -1978,24 +2057,27 @@
         <v>24</v>
       </c>
       <c r="J29" s="9" t="s">
+        <v>173</v>
+      </c>
+      <c r="K29" s="17" t="s">
         <v>174</v>
-      </c>
-      <c r="K29" s="17" t="s">
-        <v>175</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" s="7" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B30" s="3" t="s">
         <v>22</v>
       </c>
       <c r="C30" s="14" t="s">
-        <v>105</v>
+        <v>104</v>
+      </c>
+      <c r="D30" s="30" t="s">
+        <v>23</v>
       </c>
       <c r="E30" s="16" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F30" s="29">
         <v>45</v>
@@ -2004,11 +2086,14 @@
         <v>24</v>
       </c>
       <c r="J30" s="26" t="s">
+        <v>175</v>
+      </c>
+      <c r="K30" s="27" t="s">
         <v>176</v>
       </c>
-      <c r="K30" s="27" t="s">
-        <v>177</v>
-      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="D31" s="30"/>
     </row>
   </sheetData>
   <dataValidations count="2">
@@ -2034,7 +2119,7 @@
   <sheetData>
     <row r="1" spans="1:2" ht="17.25" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -2042,17 +2127,17 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -2060,7 +2145,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -2068,7 +2153,7 @@
         <v>0</v>
       </c>
       <c r="B8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -2076,7 +2161,7 @@
         <v>1</v>
       </c>
       <c r="B9" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -2084,7 +2169,7 @@
         <v>2</v>
       </c>
       <c r="B10" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
@@ -2092,7 +2177,7 @@
         <v>3</v>
       </c>
       <c r="B11" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
@@ -2100,7 +2185,7 @@
         <v>4</v>
       </c>
       <c r="B12" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
@@ -2108,7 +2193,7 @@
         <v>5</v>
       </c>
       <c r="B13" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
@@ -2116,7 +2201,7 @@
         <v>6</v>
       </c>
       <c r="B14" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
@@ -2124,7 +2209,7 @@
         <v>7</v>
       </c>
       <c r="B15" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
@@ -2132,7 +2217,7 @@
         <v>8</v>
       </c>
       <c r="B16" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
@@ -2140,7 +2225,7 @@
         <v>9</v>
       </c>
       <c r="B17" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
@@ -2148,7 +2233,7 @@
         <v>10</v>
       </c>
       <c r="B18" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
@@ -2156,18 +2241,18 @@
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="B20" t="s">
         <v>48</v>
-      </c>
-      <c r="B20" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="B21" t="s">
         <v>50</v>
-      </c>
-      <c r="B21" t="s">
-        <v>51</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix mappa maxi: corretta coord NA190 (mancava il punto decimale) + guardia coord impossibili
- NA190 aveva 408909184/142226047 (senza decimale) -> allargava la mappa al mondo
- corretto nell'xlsx: 40.8909184 / 14.2226047; dati rigenerati
- renderMap: ignora marker con lat/lng fuori range (-90..90 / -180..180)
- build-maxi-data.py: avvisa se una coord è fuori scala
- cache-buster maxi.js v6

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/maxi-impianti.xlsx
+++ b/maxi-impianti.xlsx
@@ -2093,11 +2093,15 @@
           <t>na190-1.jpg</t>
         </is>
       </c>
-      <c r="J24" s="29" t="n">
-        <v>408909184</v>
-      </c>
-      <c r="K24" s="30" t="n">
-        <v>142226047</v>
+      <c r="J24" s="29" t="inlineStr">
+        <is>
+          <t>40.8909184</t>
+        </is>
+      </c>
+      <c r="K24" s="30" t="inlineStr">
+        <is>
+          <t>14.2226047</t>
+        </is>
       </c>
       <c r="L24" s="23" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Maxi: link presentazione PDF per impianto (colonna Excel 'pdf' -> pulsante in scheda)
Aggiunta colonna 'pdf' nell'Excel e nella pipeline; il pulsante 'Vedi presentazione (PDF)' compare nella scheda solo se il link e' valorizzato. Apre in nuova scheda. i18n IT/EN/ZH.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/maxi-impianti.xlsx
+++ b/maxi-impianti.xlsx
@@ -749,7 +749,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M28"/>
+  <dimension ref="A1:O28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" style="37" min="1" max="1"/>
@@ -831,6 +831,11 @@
           <t>photo3</t>
         </is>
       </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -896,6 +901,11 @@
       <c r="M2" s="22" t="inlineStr">
         <is>
           <t>Foto 3</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Presentazione (link Drive)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Maxi: dataset ampliato a 47 impianti + foto multiple per scheda
Aggiunte foto (fino a 2 per impianto), rigenerati maxi-data.js e colonna link_web. Corretti refusi: NA02 (na02-1,jpg -> na02-1.jpg) e NA17 (na17- + file doppia estensione -> na17-1.jpg). Nessuna referenza foto rotta.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/maxi-impianti.xlsx
+++ b/maxi-impianti.xlsx
@@ -22,7 +22,7 @@
     <numFmt numFmtId="164" formatCode="_-[$€-2]\ * #.##0.0_-;\-[$€-2]\ * #.##0.0_-;_-[$€-2]\ * \-??_-"/>
     <numFmt numFmtId="165" formatCode="_-&quot;€ &quot;* #.##0.00_-;&quot;-€ &quot;* #.##0.00_-;_-&quot;€ &quot;* \-??_-;_-@_-"/>
   </numFmts>
-  <fonts count="17">
+  <fonts count="19">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -121,11 +121,23 @@
       <sz val="11"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <color rgb="FF1155CC"/>
+      <sz val="11"/>
+      <u val="single"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <sz val="10"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <color rgb="001155CC"/>
       <u val="single"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -180,6 +192,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFEE7D00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF66FF66"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -297,7 +321,7 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0"/>
     <xf numFmtId="165" fontId="10" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -381,8 +405,49 @@
     <xf numFmtId="0" fontId="8" fillId="7" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="4">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="17" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="4">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="17" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="4">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="17" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="4">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
@@ -752,7 +817,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P28"/>
+  <dimension ref="A1:P49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -961,7 +1026,7 @@
       <c r="H3" s="3" t="n"/>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>na01.jpg</t>
+          <t>na04.jpg</t>
         </is>
       </c>
       <c r="J3" s="7" t="inlineStr">
@@ -981,7 +1046,7 @@
           <t>https://drive.google.com/file/d/16vG1RTYz_ScddE7d_eqsRnU2dbDt3SRa/view?usp=drive_link</t>
         </is>
       </c>
-      <c r="P3" s="36" t="inlineStr">
+      <c r="P3" s="51" t="inlineStr">
         <is>
           <t>https://www.diessemedia.it/maxi.html#imp=NA04</t>
         </is>
@@ -1044,7 +1109,7 @@
           <t>https://drive.google.com/file/d/1yDqAyeVnIQOOv0N9Q7h7PoS-8-6djMbV/view?usp=drive_link</t>
         </is>
       </c>
-      <c r="P4" s="36" t="inlineStr">
+      <c r="P4" s="51" t="inlineStr">
         <is>
           <t>https://www.diessemedia.it/maxi.html#imp=NA05</t>
         </is>
@@ -1111,7 +1176,7 @@
           <t>https://drive.google.com/file/d/1_pZnlgOJmH_yb_HBnMEx-GBht_i0yzVz/view?usp=drive_link</t>
         </is>
       </c>
-      <c r="P5" s="36" t="inlineStr">
+      <c r="P5" s="51" t="inlineStr">
         <is>
           <t>https://www.diessemedia.it/maxi.html#imp=NA63</t>
         </is>
@@ -1174,7 +1239,7 @@
           <t>https://drive.google.com/file/d/1HfmI5m4J2SFTwVEJCmJHHJySQONbAO1b/view?usp=drive_link</t>
         </is>
       </c>
-      <c r="P6" s="36" t="inlineStr">
+      <c r="P6" s="51" t="inlineStr">
         <is>
           <t>https://www.diessemedia.it/maxi.html#imp=NA65</t>
         </is>
@@ -1206,15 +1271,15 @@
           <t>6x6 illuminato</t>
         </is>
       </c>
-      <c r="F7" s="20" t="n">
+      <c r="F7" s="50" t="n">
         <v>36</v>
       </c>
-      <c r="G7" s="19" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="I7" s="35" t="inlineStr">
+      <c r="G7" s="49" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="I7" s="31" t="inlineStr">
         <is>
           <t>na64-1.jpg</t>
         </is>
@@ -1240,7 +1305,7 @@
           <t>https://drive.google.com/file/d/1D8o9wIFWrjgf6GfDilP10zFUaph8ATAv/view?usp=sharing</t>
         </is>
       </c>
-      <c r="P7" s="36" t="inlineStr">
+      <c r="P7" s="51" t="inlineStr">
         <is>
           <t>https://www.diessemedia.it/maxi.html#imp=NA64</t>
         </is>
@@ -1272,15 +1337,15 @@
           <t>7X10 illuminato</t>
         </is>
       </c>
-      <c r="F8" s="20" t="n">
+      <c r="F8" s="50" t="n">
         <v>70</v>
       </c>
-      <c r="G8" s="19" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="I8" s="35" t="inlineStr">
+      <c r="G8" s="49" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="I8" s="31" t="inlineStr">
         <is>
           <t>na66-1.jpg</t>
         </is>
@@ -1306,7 +1371,7 @@
           <t>https://drive.google.com/file/d/1IVRloIC_Q4PKfq3crD6lGZBN-blA79on/view?usp=drive_link</t>
         </is>
       </c>
-      <c r="P8" s="36" t="inlineStr">
+      <c r="P8" s="51" t="inlineStr">
         <is>
           <t>https://www.diessemedia.it/maxi.html#imp=NA66</t>
         </is>
@@ -1338,15 +1403,15 @@
           <t>7X10 illuminato</t>
         </is>
       </c>
-      <c r="F9" s="20" t="n">
+      <c r="F9" s="50" t="n">
         <v>70</v>
       </c>
-      <c r="G9" s="19" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="I9" s="35" t="inlineStr">
+      <c r="G9" s="49" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="I9" s="31" t="inlineStr">
         <is>
           <t>na68-1.jpg</t>
         </is>
@@ -1372,7 +1437,7 @@
           <t>https://drive.google.com/file/d/1Zrx-VMiTF8AY2WcJGOUjl8_ok1kfFUuK/view?usp=drive_link</t>
         </is>
       </c>
-      <c r="P9" s="36" t="inlineStr">
+      <c r="P9" s="51" t="inlineStr">
         <is>
           <t>https://www.diessemedia.it/maxi.html#imp=NA68</t>
         </is>
@@ -1404,15 +1469,15 @@
           <t>4x9 illuminato</t>
         </is>
       </c>
-      <c r="F10" s="20" t="n">
+      <c r="F10" s="50" t="n">
         <v>36</v>
       </c>
-      <c r="G10" s="19" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="I10" s="35" t="inlineStr">
+      <c r="G10" s="49" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="I10" s="31" t="inlineStr">
         <is>
           <t>na69-1.jpg</t>
         </is>
@@ -1438,7 +1503,7 @@
           <t>https://drive.google.com/file/d/1P2GetYKby0ZKu5poZp3cjTc_5I_nnOrk/view?usp=drive_link</t>
         </is>
       </c>
-      <c r="P10" s="36" t="inlineStr">
+      <c r="P10" s="51" t="inlineStr">
         <is>
           <t>https://www.diessemedia.it/maxi.html#imp=NA69</t>
         </is>
@@ -1470,15 +1535,15 @@
           <t>7X10 illuminato</t>
         </is>
       </c>
-      <c r="F11" s="20" t="n">
+      <c r="F11" s="50" t="n">
         <v>70</v>
       </c>
-      <c r="G11" s="19" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="I11" s="35" t="inlineStr">
+      <c r="G11" s="49" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="I11" s="31" t="inlineStr">
         <is>
           <t>na67-1.jpg</t>
         </is>
@@ -1504,7 +1569,7 @@
           <t>https://drive.google.com/file/d/1UZtydQ-Ss275fV93nZSCR4GNqHCBAMXp/view?usp=drive_link</t>
         </is>
       </c>
-      <c r="P11" s="36" t="inlineStr">
+      <c r="P11" s="51" t="inlineStr">
         <is>
           <t>https://www.diessemedia.it/maxi.html#imp=NA67</t>
         </is>
@@ -1536,15 +1601,15 @@
           <t>7x7 illuminato</t>
         </is>
       </c>
-      <c r="F12" s="20" t="n">
+      <c r="F12" s="50" t="n">
         <v>49</v>
       </c>
-      <c r="G12" s="19" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="I12" s="35" t="inlineStr">
+      <c r="G12" s="49" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="I12" s="31" t="inlineStr">
         <is>
           <t>na72-1.jpg</t>
         </is>
@@ -1566,7 +1631,7 @@
           <t>https://drive.google.com/file/d/1DVTI2W9NsSPbjhvciY-PF7AbSpoUwhCW/view?usp=drive_link</t>
         </is>
       </c>
-      <c r="P12" s="36" t="inlineStr">
+      <c r="P12" s="51" t="inlineStr">
         <is>
           <t>https://www.diessemedia.it/maxi.html#imp=NA72</t>
         </is>
@@ -1598,15 +1663,15 @@
           <t>5X10 illuminato</t>
         </is>
       </c>
-      <c r="F13" s="20" t="n">
+      <c r="F13" s="50" t="n">
         <v>50</v>
       </c>
-      <c r="G13" s="19" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="I13" s="35" t="inlineStr">
+      <c r="G13" s="49" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="I13" s="31" t="inlineStr">
         <is>
           <t>na80-1.jpg</t>
         </is>
@@ -1632,7 +1697,7 @@
           <t>https://drive.google.com/file/d/1-ws2utLWp8qMT3opyPhKcB0srl3Pw617/view?usp=drive_link</t>
         </is>
       </c>
-      <c r="P13" s="36" t="inlineStr">
+      <c r="P13" s="51" t="inlineStr">
         <is>
           <t>https://www.diessemedia.it/maxi.html#imp=NA80</t>
         </is>
@@ -1664,15 +1729,15 @@
           <t>7X10 illuminato</t>
         </is>
       </c>
-      <c r="F14" s="20" t="n">
+      <c r="F14" s="50" t="n">
         <v>70</v>
       </c>
-      <c r="G14" s="19" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="I14" s="35" t="inlineStr">
+      <c r="G14" s="49" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="I14" s="31" t="inlineStr">
         <is>
           <t>na81-1.jpg</t>
         </is>
@@ -1698,7 +1763,7 @@
           <t>https://drive.google.com/file/d/14E1QiBU2qIAzVfw3uPP0Y-ihTmt6vQrd/view?usp=drive_link</t>
         </is>
       </c>
-      <c r="P14" s="36" t="inlineStr">
+      <c r="P14" s="51" t="inlineStr">
         <is>
           <t>https://www.diessemedia.it/maxi.html#imp=NA81</t>
         </is>
@@ -1730,15 +1795,15 @@
           <t>8x6 illuminato</t>
         </is>
       </c>
-      <c r="F15" s="20" t="n">
+      <c r="F15" s="50" t="n">
         <v>48</v>
       </c>
-      <c r="G15" s="19" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="I15" s="35" t="inlineStr">
+      <c r="G15" s="49" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="I15" s="31" t="inlineStr">
         <is>
           <t>na83-1.jpg</t>
         </is>
@@ -1764,7 +1829,7 @@
           <t>https://drive.google.com/file/d/1okdcJw-OkTzNXns26kQRsKJY8HuFJmdM/view?usp=drive_link</t>
         </is>
       </c>
-      <c r="P15" s="36" t="inlineStr">
+      <c r="P15" s="51" t="inlineStr">
         <is>
           <t>https://www.diessemedia.it/maxi.html#imp=NA83</t>
         </is>
@@ -1796,15 +1861,15 @@
           <t>5X10 illuminato</t>
         </is>
       </c>
-      <c r="F16" s="20" t="n">
+      <c r="F16" s="50" t="n">
         <v>50</v>
       </c>
-      <c r="G16" s="19" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="I16" s="35" t="inlineStr">
+      <c r="G16" s="49" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="I16" s="31" t="inlineStr">
         <is>
           <t>na86-1.jpg</t>
         </is>
@@ -1830,7 +1895,7 @@
           <t>https://drive.google.com/file/d/1TfShvjssHDDXQ35TT-i32b1b5NTg-VUg/view?usp=drive_link</t>
         </is>
       </c>
-      <c r="P16" s="36" t="inlineStr">
+      <c r="P16" s="51" t="inlineStr">
         <is>
           <t>https://www.diessemedia.it/maxi.html#imp=NA86</t>
         </is>
@@ -1862,15 +1927,15 @@
           <t>7X10 illuminato</t>
         </is>
       </c>
-      <c r="F17" s="20" t="n">
+      <c r="F17" s="50" t="n">
         <v>70</v>
       </c>
-      <c r="G17" s="19" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="I17" s="35" t="inlineStr">
+      <c r="G17" s="49" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="I17" s="31" t="inlineStr">
         <is>
           <t>na88-1.jpg</t>
         </is>
@@ -1896,7 +1961,7 @@
           <t>https://drive.google.com/file/d/1qJlGkmbJXGlOVqiBbyruYv72I1hHXzJh/view?usp=drive_link</t>
         </is>
       </c>
-      <c r="P17" s="36" t="inlineStr">
+      <c r="P17" s="51" t="inlineStr">
         <is>
           <t>https://www.diessemedia.it/maxi.html#imp=NA88</t>
         </is>
@@ -1928,15 +1993,15 @@
           <t>7X10 illuminato</t>
         </is>
       </c>
-      <c r="F18" s="20" t="n">
+      <c r="F18" s="50" t="n">
         <v>70</v>
       </c>
-      <c r="G18" s="19" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="I18" s="35" t="inlineStr">
+      <c r="G18" s="49" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="I18" s="31" t="inlineStr">
         <is>
           <t>na87-1.jpg</t>
         </is>
@@ -1962,7 +2027,7 @@
           <t>https://drive.google.com/file/d/1mCwKGFtJqE-oKLf9MpSaVk37JhpXu50h/view?usp=drive_link</t>
         </is>
       </c>
-      <c r="P18" s="36" t="inlineStr">
+      <c r="P18" s="51" t="inlineStr">
         <is>
           <t>https://www.diessemedia.it/maxi.html#imp=NA87</t>
         </is>
@@ -1994,15 +2059,15 @@
           <t>5X10  illuminato</t>
         </is>
       </c>
-      <c r="F19" s="20" t="n">
+      <c r="F19" s="50" t="n">
         <v>50</v>
       </c>
-      <c r="G19" s="19" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="I19" s="35" t="inlineStr">
+      <c r="G19" s="49" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="I19" s="31" t="inlineStr">
         <is>
           <t>na95-1.jpg</t>
         </is>
@@ -2028,7 +2093,7 @@
           <t>https://drive.google.com/file/d/1zqJA_3FH4k8WJYwdZ6DY0RB_HKzRAB_s/view?usp=sharing</t>
         </is>
       </c>
-      <c r="P19" s="36" t="inlineStr">
+      <c r="P19" s="51" t="inlineStr">
         <is>
           <t>https://www.diessemedia.it/maxi.html#imp=NA95</t>
         </is>
@@ -2060,10 +2125,10 @@
           <t>5X8 luminoso</t>
         </is>
       </c>
-      <c r="F20" s="20" t="n">
+      <c r="F20" s="50" t="n">
         <v>40</v>
       </c>
-      <c r="G20" s="19" t="inlineStr">
+      <c r="G20" s="49" t="inlineStr">
         <is>
           <t>si</t>
         </is>
@@ -2094,7 +2159,7 @@
           <t>https://drive.google.com/file/d/1LvtXYG5yNk7lCyMX_FPwBjBf0bDbdq5N/view?usp=drive_link</t>
         </is>
       </c>
-      <c r="P20" s="36" t="inlineStr">
+      <c r="P20" s="51" t="inlineStr">
         <is>
           <t>https://www.diessemedia.it/maxi.html#imp=NA91</t>
         </is>
@@ -2126,10 +2191,10 @@
           <t>7x9 illuminato</t>
         </is>
       </c>
-      <c r="F21" s="20" t="n">
+      <c r="F21" s="50" t="n">
         <v>63</v>
       </c>
-      <c r="G21" s="19" t="inlineStr">
+      <c r="G21" s="49" t="inlineStr">
         <is>
           <t>si</t>
         </is>
@@ -2160,7 +2225,7 @@
           <t>https://drive.google.com/file/d/1uItwka6i5KFoxBVyvzzXddUv7AQqT0OT/view?usp=drive_link</t>
         </is>
       </c>
-      <c r="P21" s="36" t="inlineStr">
+      <c r="P21" s="51" t="inlineStr">
         <is>
           <t>https://www.diessemedia.it/maxi.html#imp=NA92</t>
         </is>
@@ -2192,10 +2257,10 @@
           <t>6X6  illuminato</t>
         </is>
       </c>
-      <c r="F22" s="20" t="n">
+      <c r="F22" s="50" t="n">
         <v>36</v>
       </c>
-      <c r="G22" s="19" t="inlineStr">
+      <c r="G22" s="49" t="inlineStr">
         <is>
           <t>si</t>
         </is>
@@ -2222,7 +2287,7 @@
           <t>https://drive.google.com/file/d/1P3uijUwLYBVchnpBdZHCUcoA3nL4mURx/view?usp=sharing</t>
         </is>
       </c>
-      <c r="P22" s="36" t="inlineStr">
+      <c r="P22" s="51" t="inlineStr">
         <is>
           <t>https://www.diessemedia.it/maxi.html#imp=NA93</t>
         </is>
@@ -2254,10 +2319,10 @@
           <t>6x8 illuminato</t>
         </is>
       </c>
-      <c r="F23" s="20" t="n">
+      <c r="F23" s="50" t="n">
         <v>48</v>
       </c>
-      <c r="G23" s="19" t="inlineStr">
+      <c r="G23" s="49" t="inlineStr">
         <is>
           <t>si</t>
         </is>
@@ -2288,7 +2353,7 @@
           <t>https://drive.google.com/file/d/1ShkIPgc8suaDQTiWQMCz7rtt4-LVx7iU/view?usp=drive_link</t>
         </is>
       </c>
-      <c r="P23" s="36" t="inlineStr">
+      <c r="P23" s="51" t="inlineStr">
         <is>
           <t>https://www.diessemedia.it/maxi.html#imp=NA89</t>
         </is>
@@ -2320,10 +2385,10 @@
           <t>8X12 illuminato</t>
         </is>
       </c>
-      <c r="F24" s="20" t="n">
+      <c r="F24" s="50" t="n">
         <v>96</v>
       </c>
-      <c r="G24" s="19" t="inlineStr">
+      <c r="G24" s="49" t="inlineStr">
         <is>
           <t>si</t>
         </is>
@@ -2354,7 +2419,7 @@
           <t>https://drive.google.com/file/d/1DIPFK2DsZATvstk4Nfz0gkYHqxgmMKIl/view?usp=drive_link</t>
         </is>
       </c>
-      <c r="P24" s="36" t="inlineStr">
+      <c r="P24" s="51" t="inlineStr">
         <is>
           <t>https://www.diessemedia.it/maxi.html#imp=NA190</t>
         </is>
@@ -2386,10 +2451,10 @@
           <t>8X14 illuminato</t>
         </is>
       </c>
-      <c r="F25" s="20" t="n">
+      <c r="F25" s="50" t="n">
         <v>112</v>
       </c>
-      <c r="G25" s="19" t="inlineStr">
+      <c r="G25" s="49" t="inlineStr">
         <is>
           <t>si</t>
         </is>
@@ -2411,7 +2476,7 @@
           <t>https://drive.google.com/file/d/1qBGa-lPOtAlGznIwGPc7jFWoQPmatveK/view?usp=sharing</t>
         </is>
       </c>
-      <c r="P25" s="36" t="inlineStr">
+      <c r="P25" s="51" t="inlineStr">
         <is>
           <t>https://www.diessemedia.it/maxi.html#imp=NA30</t>
         </is>
@@ -2443,7 +2508,7 @@
           <t>8X14 illuminato</t>
         </is>
       </c>
-      <c r="F26" s="20" t="n">
+      <c r="F26" s="50" t="n">
         <v>112</v>
       </c>
       <c r="G26" t="inlineStr">
@@ -2477,7 +2542,7 @@
           <t>https://drive.google.com/file/d/11ksiqfCg7x3chwOC00PHi2d0SwGaa7lz/view?usp=sharing</t>
         </is>
       </c>
-      <c r="P26" s="36" t="inlineStr">
+      <c r="P26" s="51" t="inlineStr">
         <is>
           <t>https://www.diessemedia.it/maxi.html#imp=NA40</t>
         </is>
@@ -2509,7 +2574,7 @@
           <t>6x12 illuminato</t>
         </is>
       </c>
-      <c r="F27" s="20" t="n">
+      <c r="F27" s="50" t="n">
         <v>70</v>
       </c>
       <c r="G27" t="inlineStr">
@@ -2543,7 +2608,7 @@
           <t>https://drive.google.com/file/d/1B_VLsKhDSVovcVH4OYf4ya8-NSSJvmN-/view?usp=sharing</t>
         </is>
       </c>
-      <c r="P27" s="36" t="inlineStr">
+      <c r="P27" s="51" t="inlineStr">
         <is>
           <t>https://www.diessemedia.it/maxi.html#imp=NA84</t>
         </is>
@@ -2555,7 +2620,7 @@
           <t>NA120</t>
         </is>
       </c>
-      <c r="B28" s="19" t="inlineStr">
+      <c r="B28" s="49" t="inlineStr">
         <is>
           <t>Napoli</t>
         </is>
@@ -2575,7 +2640,7 @@
           <t>10x12 illuminato</t>
         </is>
       </c>
-      <c r="F28" s="20" t="n">
+      <c r="F28" s="50" t="n">
         <v>120</v>
       </c>
       <c r="G28" t="inlineStr">
@@ -2598,7 +2663,7 @@
           <t>14.2264429</t>
         </is>
       </c>
-      <c r="L28" s="19" t="inlineStr">
+      <c r="L28" s="49" t="inlineStr">
         <is>
           <t>na120-2.jpg</t>
         </is>
@@ -2608,9 +2673,1266 @@
           <t>https://drive.google.com/file/d/1xXT2OPWld2_Lp_rAYi0_wQf0wva57TT3/view?usp=drive_link</t>
         </is>
       </c>
-      <c r="P28" s="36" t="inlineStr">
+      <c r="P28" s="51" t="inlineStr">
         <is>
           <t>https://www.diessemedia.it/maxi.html#imp=NA120</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="36" t="inlineStr">
+        <is>
+          <t>NA01</t>
+        </is>
+      </c>
+      <c r="B29" s="49" t="inlineStr">
+        <is>
+          <t>Napoli</t>
+        </is>
+      </c>
+      <c r="C29" s="39" t="inlineStr">
+        <is>
+          <t>P.ZZA GARIBALDI FRONTE CORSO A. LUCCI - STAZIONE CENTRALE</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Facciata</t>
+        </is>
+      </c>
+      <c r="E29" s="39" t="inlineStr">
+        <is>
+          <t>17X8 illuminato</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>na01-1.jpg</t>
+        </is>
+      </c>
+      <c r="J29" s="42" t="inlineStr">
+        <is>
+          <t>40.852507</t>
+        </is>
+      </c>
+      <c r="K29" s="42" t="inlineStr">
+        <is>
+          <t>14.271571</t>
+        </is>
+      </c>
+      <c r="L29" s="49" t="inlineStr">
+        <is>
+          <t>na01-2.jpg</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1Ze99d7OndJiHONdJFjvBrhxfm-ZUEGBj/view?usp=drive_link</t>
+        </is>
+      </c>
+      <c r="P29" s="51" t="inlineStr">
+        <is>
+          <t>https://www.diessemedia.it/maxi.html#imp=NA01</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="37" t="inlineStr">
+        <is>
+          <t>NA02</t>
+        </is>
+      </c>
+      <c r="B30" s="49" t="inlineStr">
+        <is>
+          <t>Napoli</t>
+        </is>
+      </c>
+      <c r="C30" s="39" t="inlineStr">
+        <is>
+          <t>P.ZZA GARIBALDI FRONTE CORSO  UMBERTO - STAZIONE CENTRALE</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Facciata</t>
+        </is>
+      </c>
+      <c r="E30" s="39" t="inlineStr">
+        <is>
+          <t>14X6 illuminato</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>na02-1.jpg</t>
+        </is>
+      </c>
+      <c r="J30" s="43" t="inlineStr">
+        <is>
+          <t>40.853170</t>
+        </is>
+      </c>
+      <c r="K30" s="43" t="inlineStr">
+        <is>
+          <t>14.270822</t>
+        </is>
+      </c>
+      <c r="L30" s="50" t="inlineStr">
+        <is>
+          <t>na02-2.jpg</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1dMLz8vu4fDBJgTwc-EI2XnPrruwlwRGl/view?usp=drive_link</t>
+        </is>
+      </c>
+      <c r="P30" s="51" t="inlineStr">
+        <is>
+          <t>https://www.diessemedia.it/maxi.html#imp=NA02</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="38" t="inlineStr">
+        <is>
+          <t>NA32</t>
+        </is>
+      </c>
+      <c r="B31" s="49" t="inlineStr">
+        <is>
+          <t>Napoli</t>
+        </is>
+      </c>
+      <c r="C31" s="39" t="inlineStr">
+        <is>
+          <t>P.ZZA GARIBALDI FR.HOTEL TERMINUS -STAZIONE CENTRALE</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Facciata</t>
+        </is>
+      </c>
+      <c r="E31" s="39" t="inlineStr">
+        <is>
+          <t>14X4 illuminato</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>na32-1.jpg</t>
+        </is>
+      </c>
+      <c r="J31" s="17" t="inlineStr">
+        <is>
+          <t>40.852521</t>
+        </is>
+      </c>
+      <c r="K31" s="17" t="inlineStr">
+        <is>
+          <t>14.270780</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/12ZZ8slp22tMFC_P7G_CArH8UrY8JWfLW/view?usp=drive_link</t>
+        </is>
+      </c>
+      <c r="P31" s="51" t="inlineStr">
+        <is>
+          <t>https://www.diessemedia.it/maxi.html#imp=NA32</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="37" t="inlineStr">
+        <is>
+          <t>NA03</t>
+        </is>
+      </c>
+      <c r="B32" s="49" t="inlineStr">
+        <is>
+          <t>Napoli</t>
+        </is>
+      </c>
+      <c r="C32" s="39" t="inlineStr">
+        <is>
+          <t>VIA C. ROSARROL DIREZIONE VIA FORIA</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Facciata</t>
+        </is>
+      </c>
+      <c r="E32" s="39" t="inlineStr">
+        <is>
+          <t>7X8 illuminato</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>na03-1.jpg</t>
+        </is>
+      </c>
+      <c r="J32" s="44" t="inlineStr">
+        <is>
+          <t>40.855482</t>
+        </is>
+      </c>
+      <c r="K32" s="44" t="inlineStr">
+        <is>
+          <t>14.265060</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1-bSXxZh7gRSM7FzagRSVyD3tzCL8K19c/view?usp=drive_link</t>
+        </is>
+      </c>
+      <c r="P32" s="51" t="inlineStr">
+        <is>
+          <t>https://www.diessemedia.it/maxi.html#imp=NA03</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="36" t="inlineStr">
+        <is>
+          <t>NA09</t>
+        </is>
+      </c>
+      <c r="B33" s="49" t="inlineStr">
+        <is>
+          <t>Napoli</t>
+        </is>
+      </c>
+      <c r="C33" s="39" t="inlineStr">
+        <is>
+          <t>VIALE F. RUFFO DI CALABRIA USCITA AEREOPORTO CAPODICHINO</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Facciata</t>
+        </is>
+      </c>
+      <c r="E33" s="39" t="inlineStr">
+        <is>
+          <t>8x4 illuminato</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>na09-1.jpg</t>
+        </is>
+      </c>
+      <c r="J33" s="44" t="inlineStr">
+        <is>
+          <t>40.874682</t>
+        </is>
+      </c>
+      <c r="K33" s="44" t="inlineStr">
+        <is>
+          <t>14.285230</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>na09-2.jpg</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1_dDzdcm1SW2BRHJ4REEXt63KhKC7TTwO/view?usp=drive_link</t>
+        </is>
+      </c>
+      <c r="P33" s="51" t="inlineStr">
+        <is>
+          <t>https://www.diessemedia.it/maxi.html#imp=NA09</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="37" t="inlineStr">
+        <is>
+          <t>NA16</t>
+        </is>
+      </c>
+      <c r="B34" s="49" t="inlineStr">
+        <is>
+          <t>Napoli</t>
+        </is>
+      </c>
+      <c r="C34" s="39" t="inlineStr">
+        <is>
+          <t>VIA NUOVA POGGIOREALE INCR. VIA AUSILIO dir.uscita città</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Facciata</t>
+        </is>
+      </c>
+      <c r="E34" s="39" t="inlineStr">
+        <is>
+          <t>8x4 illuminato</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>na16-1.jpg</t>
+        </is>
+      </c>
+      <c r="J34" s="44" t="inlineStr">
+        <is>
+          <t>40.863074</t>
+        </is>
+      </c>
+      <c r="K34" s="44" t="inlineStr">
+        <is>
+          <t>14.283740</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1L_KUat2119meWNPJmzPXrF7gvf0e5Qvk/view?usp=drive_link</t>
+        </is>
+      </c>
+      <c r="P34" s="51" t="inlineStr">
+        <is>
+          <t>https://www.diessemedia.it/maxi.html#imp=NA16</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="37" t="inlineStr">
+        <is>
+          <t>NA13</t>
+        </is>
+      </c>
+      <c r="B35" s="49" t="inlineStr">
+        <is>
+          <t>Napoli</t>
+        </is>
+      </c>
+      <c r="C35" s="39" t="inlineStr">
+        <is>
+          <t>VIA DOMENICO FONTANA INC.  A. ROCCO DIREZIONE PIAZZA MUZII</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Facciata</t>
+        </is>
+      </c>
+      <c r="E35" s="40" t="inlineStr">
+        <is>
+          <t>6X9 illuminato</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>na13-1.jpg</t>
+        </is>
+      </c>
+      <c r="J35" s="44" t="inlineStr">
+        <is>
+          <t>40.854590</t>
+        </is>
+      </c>
+      <c r="K35" s="44" t="inlineStr">
+        <is>
+          <t>14.228845</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1qmPB9seFCrh8sNkIHPcT3dyM4_EB5_w4/view?usp=drive_link</t>
+        </is>
+      </c>
+      <c r="P35" s="51" t="inlineStr">
+        <is>
+          <t>https://www.diessemedia.it/maxi.html#imp=NA13</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="37" t="inlineStr">
+        <is>
+          <t>NA11</t>
+        </is>
+      </c>
+      <c r="B36" s="49" t="inlineStr">
+        <is>
+          <t>Napoli</t>
+        </is>
+      </c>
+      <c r="C36" s="39" t="inlineStr">
+        <is>
+          <t>TANGENZIALE ALTEZZA SVINCOLO  CAPODICHINO DIREZIONE CENTRO</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Facciata</t>
+        </is>
+      </c>
+      <c r="E36" s="41" t="inlineStr">
+        <is>
+          <t>11X4 illuminato</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>na11-1.jpg</t>
+        </is>
+      </c>
+      <c r="J36" s="44" t="inlineStr">
+        <is>
+          <t>40.874769</t>
+        </is>
+      </c>
+      <c r="K36" s="44" t="inlineStr">
+        <is>
+          <t>14.288231</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>na11-2.jpg</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1cC3aKjNdAbamecgbWj4WkiUaB4jwf6BZ/view?usp=drive_link</t>
+        </is>
+      </c>
+      <c r="P36" s="51" t="inlineStr">
+        <is>
+          <t>https://www.diessemedia.it/maxi.html#imp=NA11</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="37" t="inlineStr">
+        <is>
+          <t>NA17</t>
+        </is>
+      </c>
+      <c r="B37" s="49" t="inlineStr">
+        <is>
+          <t>Napoli</t>
+        </is>
+      </c>
+      <c r="C37" s="39" t="inlineStr">
+        <is>
+          <t>TANGENZIALE SV. CAPODICHINO  DIREZIONE CENTRO CITTA'</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Facciata</t>
+        </is>
+      </c>
+      <c r="E37" s="39" t="inlineStr">
+        <is>
+          <t>8x4 illuminato</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>na17-1.jpg</t>
+        </is>
+      </c>
+      <c r="J37" s="45" t="inlineStr">
+        <is>
+          <t>40.874072</t>
+        </is>
+      </c>
+      <c r="K37" s="45" t="inlineStr">
+        <is>
+          <t>14.287265</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1UboUIwvETUkzomjvAJs7wjkZlwrI-hPz/view?usp=drive_link</t>
+        </is>
+      </c>
+      <c r="P37" s="51" t="inlineStr">
+        <is>
+          <t>https://www.diessemedia.it/maxi.html#imp=NA17</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="37" t="inlineStr">
+        <is>
+          <t>NA14</t>
+        </is>
+      </c>
+      <c r="B38" s="49" t="inlineStr">
+        <is>
+          <t>Napoli</t>
+        </is>
+      </c>
+      <c r="C38" s="39" t="inlineStr">
+        <is>
+          <t>VIA MASCAGNI INCROCIO VIA DE NARDIS DIREZIONE VIA CILEA</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Facciata</t>
+        </is>
+      </c>
+      <c r="E38" s="40" t="inlineStr">
+        <is>
+          <t>6x7 illuminato</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>na14-1.jpg</t>
+        </is>
+      </c>
+      <c r="J38" s="46" t="inlineStr">
+        <is>
+          <t>40.844741</t>
+        </is>
+      </c>
+      <c r="K38" s="46" t="inlineStr">
+        <is>
+          <t>14.221057</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1VUL0qzQO1PsINjrF519-55fk9mI2TQm9/view?usp=drive_link</t>
+        </is>
+      </c>
+      <c r="P38" s="51" t="inlineStr">
+        <is>
+          <t>https://www.diessemedia.it/maxi.html#imp=NA14</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="37" t="inlineStr">
+        <is>
+          <t>NA06</t>
+        </is>
+      </c>
+      <c r="B39" s="49" t="inlineStr">
+        <is>
+          <t>Napoli</t>
+        </is>
+      </c>
+      <c r="C39" s="39" t="inlineStr">
+        <is>
+          <t>VIA GIAMBATTISTA MARINO ANG. J. DE GENNARO - STADIO MARADONA</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Facciata</t>
+        </is>
+      </c>
+      <c r="E39" s="39" t="inlineStr">
+        <is>
+          <t>6x6 illuminato</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>na06-1.jpg</t>
+        </is>
+      </c>
+      <c r="J39" s="44" t="inlineStr">
+        <is>
+          <t>40.828856</t>
+        </is>
+      </c>
+      <c r="K39" s="44" t="inlineStr">
+        <is>
+          <t>14.196072</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>na06-2.jpg</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1f-tBKHWbm3RulZkiGC_Xy0V6lplfMKlQ/view?usp=drive_link</t>
+        </is>
+      </c>
+      <c r="P39" s="51" t="inlineStr">
+        <is>
+          <t>https://www.diessemedia.it/maxi.html#imp=NA06</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="37" t="inlineStr">
+        <is>
+          <t>NA10</t>
+        </is>
+      </c>
+      <c r="B40" s="49" t="inlineStr">
+        <is>
+          <t>Napoli</t>
+        </is>
+      </c>
+      <c r="C40" s="39" t="inlineStr">
+        <is>
+          <t>TANGENZIALE ALTEZZA SVINCOLO CAPODICHINO DIREZIONE  AUTOSTRADE</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Facciata</t>
+        </is>
+      </c>
+      <c r="E40" s="41" t="inlineStr">
+        <is>
+          <t>9X4.5 illuminato</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>na10-1.jpg</t>
+        </is>
+      </c>
+      <c r="J40" s="44" t="inlineStr">
+        <is>
+          <t>40.875306</t>
+        </is>
+      </c>
+      <c r="K40" s="44" t="inlineStr">
+        <is>
+          <t>14.288729</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>na10-2.jpg</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1BAdv7cWbPWtiRHO7E8iub7w_y6h8o-fv/view?usp=drive_link</t>
+        </is>
+      </c>
+      <c r="P40" s="51" t="inlineStr">
+        <is>
+          <t>https://www.diessemedia.it/maxi.html#imp=NA10</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="37" t="inlineStr">
+        <is>
+          <t>NA07</t>
+        </is>
+      </c>
+      <c r="B41" s="49" t="inlineStr">
+        <is>
+          <t>Napoli</t>
+        </is>
+      </c>
+      <c r="C41" s="47" t="inlineStr">
+        <is>
+          <t>V.LE MICHELANGELO DIREZIONE PIAZZA LEONARDO</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Facciata</t>
+        </is>
+      </c>
+      <c r="E41" s="47" t="inlineStr">
+        <is>
+          <t>7X10 illuminato</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>na07-1.jpg</t>
+        </is>
+      </c>
+      <c r="J41" s="44" t="inlineStr">
+        <is>
+          <t>40.847880</t>
+        </is>
+      </c>
+      <c r="K41" s="44" t="inlineStr">
+        <is>
+          <t>14.233800</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>na07-2.jpg</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1lEAVJbr9sbTwOyx99WPGE5yr8DUu-5qO/view?usp=drive_link</t>
+        </is>
+      </c>
+      <c r="P41" s="51" t="inlineStr">
+        <is>
+          <t>https://www.diessemedia.it/maxi.html#imp=NA07</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="37" t="inlineStr">
+        <is>
+          <t>NA08</t>
+        </is>
+      </c>
+      <c r="B42" s="49" t="inlineStr">
+        <is>
+          <t>Napoli</t>
+        </is>
+      </c>
+      <c r="C42" s="39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VIA S. GENNARO AD ANTIGNANO INCR. VIA MERLIANI DIR. PIAZZA DEGLI ARTISTI </t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Facciata</t>
+        </is>
+      </c>
+      <c r="E42" s="39" t="inlineStr">
+        <is>
+          <t>6X9 illuminato</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>na08-1.jpg</t>
+        </is>
+      </c>
+      <c r="J42" s="46" t="inlineStr">
+        <is>
+          <t>40.847214</t>
+        </is>
+      </c>
+      <c r="K42" s="46" t="inlineStr">
+        <is>
+          <t>14.229604</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1eDarPFYfUM_qcZOXxtMlDLLYPf47AENQ/view?usp=drive_link</t>
+        </is>
+      </c>
+      <c r="P42" s="51" t="inlineStr">
+        <is>
+          <t>https://www.diessemedia.it/maxi.html#imp=NA08</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="36" t="inlineStr">
+        <is>
+          <t>NA15</t>
+        </is>
+      </c>
+      <c r="B43" s="49" t="inlineStr">
+        <is>
+          <t>Napoli</t>
+        </is>
+      </c>
+      <c r="C43" s="39" t="inlineStr">
+        <is>
+          <t>VIA TASSO DIREZIONE INCROCIO VIA ANIELLO FALCONE</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Facciata</t>
+        </is>
+      </c>
+      <c r="E43" s="39" t="inlineStr">
+        <is>
+          <t>6x9 illuminato</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>na15-1.jpg</t>
+        </is>
+      </c>
+      <c r="J43" s="44" t="inlineStr">
+        <is>
+          <t>40.838444</t>
+        </is>
+      </c>
+      <c r="K43" s="44" t="inlineStr">
+        <is>
+          <t>14.223576</t>
+        </is>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1D-c2BC1E2rfX8UZ-SgDupmSy9CqrIiNL/view?usp=drive_link</t>
+        </is>
+      </c>
+      <c r="P43" s="51" t="inlineStr">
+        <is>
+          <t>https://www.diessemedia.it/maxi.html#imp=NA15</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="37" t="inlineStr">
+        <is>
+          <t>NA18</t>
+        </is>
+      </c>
+      <c r="B44" s="49" t="inlineStr">
+        <is>
+          <t>Napoli</t>
+        </is>
+      </c>
+      <c r="C44" s="39" t="inlineStr">
+        <is>
+          <t>VIA SALOMONE ROTATORIA USCITA AEREOPORTO INGRESSO TANGENZIALE CAPODICHINO E INGR. AUTOSTRADE</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Facciata</t>
+        </is>
+      </c>
+      <c r="E44" s="41" t="inlineStr">
+        <is>
+          <t>8x4 illuminato</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>na18-1.jpg</t>
+        </is>
+      </c>
+      <c r="J44" s="45" t="inlineStr">
+        <is>
+          <t>40.873807</t>
+        </is>
+      </c>
+      <c r="K44" s="45" t="inlineStr">
+        <is>
+          <t>14.286437</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>na18-2.jpg</t>
+        </is>
+      </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1DZYTUi22pOGkUP3MSDksJl291FbRhO19/view?usp=drive_link</t>
+        </is>
+      </c>
+      <c r="P44" s="51" t="inlineStr">
+        <is>
+          <t>https://www.diessemedia.it/maxi.html#imp=NA18</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="38" t="inlineStr">
+        <is>
+          <t>NA26</t>
+        </is>
+      </c>
+      <c r="B45" s="49" t="inlineStr">
+        <is>
+          <t>Napoli</t>
+        </is>
+      </c>
+      <c r="C45" s="39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VIA NUOVA AGNANO ANGOLO GIOCHI DEL MEDITERRANEO  </t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Facciata</t>
+        </is>
+      </c>
+      <c r="E45" s="39" t="inlineStr">
+        <is>
+          <t>6x9 illuminato</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>na26-1.jpg</t>
+        </is>
+      </c>
+      <c r="J45" s="45" t="inlineStr">
+        <is>
+          <t>40.820430</t>
+        </is>
+      </c>
+      <c r="K45" s="45" t="inlineStr">
+        <is>
+          <t>14.174702</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>na26-2.jpg</t>
+        </is>
+      </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1vS0h0SqJvD7tzLaLmkq_7kUCMKit9ns5/view?usp=drive_link</t>
+        </is>
+      </c>
+      <c r="P45" s="51" t="inlineStr">
+        <is>
+          <t>https://www.diessemedia.it/maxi.html#imp=NA26</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="37" t="inlineStr">
+        <is>
+          <t>NA22</t>
+        </is>
+      </c>
+      <c r="B46" s="49" t="inlineStr">
+        <is>
+          <t>Napoli</t>
+        </is>
+      </c>
+      <c r="C46" s="39" t="inlineStr">
+        <is>
+          <t>VIA VOLTA  - MARINA DIR.CENTRO</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Facciata</t>
+        </is>
+      </c>
+      <c r="E46" s="40" t="inlineStr">
+        <is>
+          <t>9x4,5 illuminato</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>na22-1.jpg</t>
+        </is>
+      </c>
+      <c r="J46" s="45" t="inlineStr">
+        <is>
+          <t>40.845043</t>
+        </is>
+      </c>
+      <c r="K46" s="45" t="inlineStr">
+        <is>
+          <t>14.281764</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>na22-2.jpg</t>
+        </is>
+      </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1TAA_0QMeeSx9FxPytHfIX8JPGvieg9_t/view?usp=drive_link</t>
+        </is>
+      </c>
+      <c r="P46" s="51" t="inlineStr">
+        <is>
+          <t>https://www.diessemedia.it/maxi.html#imp=NA22</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="38" t="inlineStr">
+        <is>
+          <t>NA23</t>
+        </is>
+      </c>
+      <c r="B47" s="49" t="inlineStr">
+        <is>
+          <t>Napoli</t>
+        </is>
+      </c>
+      <c r="C47" s="39" t="inlineStr">
+        <is>
+          <t>VIA CINTHIA FRONTE INGRESSO TANGENZIALE FUORIGROTTA</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Facciata</t>
+        </is>
+      </c>
+      <c r="E47" s="39" t="inlineStr">
+        <is>
+          <t>8x4 illuminato</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>na23-1.jpg</t>
+        </is>
+      </c>
+      <c r="J47" s="45" t="inlineStr">
+        <is>
+          <t>40.834053</t>
+        </is>
+      </c>
+      <c r="K47" s="45" t="inlineStr">
+        <is>
+          <t>14.190913</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>na23-2.jpg</t>
+        </is>
+      </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/17XPU8tk31w34w1FSazSzY7lTmrLVJ2D1/view?usp=drive_link</t>
+        </is>
+      </c>
+      <c r="P47" s="51" t="inlineStr">
+        <is>
+          <t>https://www.diessemedia.it/maxi.html#imp=NA23</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="36" t="inlineStr">
+        <is>
+          <t>NA24</t>
+        </is>
+      </c>
+      <c r="B48" s="49" t="inlineStr">
+        <is>
+          <t>Napoli</t>
+        </is>
+      </c>
+      <c r="C48" s="39" t="inlineStr">
+        <is>
+          <t>CORSO NOVARA ALT. VIA NAZIONALE DIR. PIAZZA GARIBALDI STAZIONE CENTRALE</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Facciata</t>
+        </is>
+      </c>
+      <c r="E48" s="39" t="inlineStr">
+        <is>
+          <t>6x9 illuminato</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>na24-1.jpg</t>
+        </is>
+      </c>
+      <c r="J48" s="48" t="inlineStr">
+        <is>
+          <t>40.856386</t>
+        </is>
+      </c>
+      <c r="K48" s="48" t="inlineStr">
+        <is>
+          <t>14.271022</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>na24-2.jpg</t>
+        </is>
+      </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1oDUDxhu0tmAy-Fb96Bm097gSwrbBMmso/view?usp=drive_link</t>
+        </is>
+      </c>
+      <c r="P48" s="51" t="inlineStr">
+        <is>
+          <t>https://www.diessemedia.it/maxi.html#imp=NA24</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="38" t="inlineStr">
+        <is>
+          <t>NA25</t>
+        </is>
+      </c>
+      <c r="B49" s="49" t="inlineStr">
+        <is>
+          <t>Napoli</t>
+        </is>
+      </c>
+      <c r="C49" s="39" t="inlineStr">
+        <is>
+          <t>VIA GIUSTINIANO MT 100 ROTATORIA USC. TANGENZIALE VIA EPOMEO</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Facciata</t>
+        </is>
+      </c>
+      <c r="E49" s="39" t="inlineStr">
+        <is>
+          <t>6x9 illuminato</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>na25-1.jpg</t>
+        </is>
+      </c>
+      <c r="J49" s="45" t="inlineStr">
+        <is>
+          <t>40.842523</t>
+        </is>
+      </c>
+      <c r="K49" s="45" t="inlineStr">
+        <is>
+          <t>14.206922</t>
+        </is>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/11-LKJADVG19BuwOtan7CnYbsTBeD-zpk/view?usp=drive_link</t>
+        </is>
+      </c>
+      <c r="P49" s="51" t="inlineStr">
+        <is>
+          <t>https://www.diessemedia.it/maxi.html#imp=NA25</t>
         </is>
       </c>
     </row>
@@ -2650,6 +3972,27 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P26" r:id="rId24"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P27" r:id="rId25"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P28" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P29" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P30" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P31" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P32" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P33" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P34" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P35" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P36" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P37" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P38" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P39" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P40" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P41" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P42" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P43" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P44" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P45" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P46" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P47" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P48" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P49" r:id="rId47"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" scale="48" fitToHeight="0"/>

</xml_diff>